<commit_message>
Update reports 2026-10-20 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-20.xlsx
+++ b/gex_pivot_levels_2026-10-20.xlsx
@@ -610,12 +610,12 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>-$5.45M</t>
+          <t>-$7.16M</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>+$5.86M</t>
+          <t>+$7.69M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>-$10.97M</t>
+          <t>-$13.85M</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$15.57M</t>
+          <t>+$19.64M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -701,12 +701,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>-$14.25M</t>
+          <t>-$17.39M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$21.06M</t>
+          <t>+$25.70M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>-$6.88M</t>
+          <t>-$7.13M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$33.17M</t>
+          <t>+$34.39M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -858,12 +858,12 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>-$3.35M</t>
+          <t>-$3.27M</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>+$18.88M</t>
+          <t>+$18.43M</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -920,12 +920,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>+$20.37M</t>
+          <t>+$16.76M</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>+$28.79M</t>
+          <t>+$23.69M</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -949,12 +949,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>+$22.60M</t>
+          <t>+$17.48M</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>+$26.22M</t>
+          <t>+$20.27M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1015,12 +1015,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$6.66M</t>
+          <t>+$4.52M</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>+$43.39M</t>
+          <t>+$29.44M</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -3242,76 +3242,76 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
-        <v>7803.52</v>
-      </c>
-      <c r="C2" s="5" t="n">
-        <v>7750</v>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="B2" s="2" t="n">
+        <v>7779.57</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>770</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>+$12.55M</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>+$34.79M</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>7753.52</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>7700</v>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>+$6.66M</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>+$43.39M</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>-$7.13M</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>+$34.39M</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>7779.57</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>770</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>+$12.55M</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>+$34.79M</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -3320,24 +3320,24 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>7753.52</v>
+        <v>7803.52</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>7700</v>
+        <v>7750</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>-$6.88M</t>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>+$4.52M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>+$33.17M</t>
+          <t>+$29.44M</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -3348,38 +3348,42 @@
       <c r="H4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>7783.52</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>7730</v>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="B5" s="2" t="n">
+        <v>7713.52</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>7660</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>+$20.37M</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>+$28.79M</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>-$17.39M</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>+$25.70M</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -3388,36 +3392,32 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>7788.52</v>
+        <v>7809.67</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>7735</v>
+        <v>773</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>+$22.60M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>-$622.23K</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>+$26.22M</t>
+          <t>+$25.43M</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3426,24 +3426,24 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7809.67</v>
+        <v>7783.52</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>773</v>
+        <v>7730</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>-$622.23K</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>+$16.76M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>+$25.43M</t>
+          <t>+$23.69M</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -3492,42 +3492,38 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
-        <v>7713.52</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>7660</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>-$14.25M</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>+$21.06M</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="B9" s="5" t="n">
+        <v>7759.5</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>768</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>+$1.12M</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>+$21.00M</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -3536,104 +3532,108 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>7759.5</v>
+        <v>7788.52</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>768</v>
+        <v>7735</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>+$1.12M</t>
+          <t>+$17.48M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>+$21.00M</t>
+          <t>+$20.27M</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7703.52</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>7650</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>-$13.85M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>+$19.64M</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B12" s="2" t="n">
         <v>29780.67</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C12" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>+$12.34M</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>+$19.41M</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>7763.52</v>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>7710</v>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>-$3.35M</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>+$18.88M</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -3642,36 +3642,32 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>7729.4</v>
+        <v>7763.52</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>765</v>
+        <v>7710</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>+$2.97M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>-$3.27M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>+$18.29M</t>
+          <t>+$18.43M</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -3680,32 +3676,36 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>7703.52</v>
+        <v>7729.4</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>7650</v>
+        <v>765</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>-$10.97M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>+$2.97M</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>+$15.57M</t>
+          <t>+$18.29M</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -4088,76 +4088,76 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B25" s="5" t="n">
+        <v>7653.52</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>7600</v>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>-$7.16M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>+$7.69M</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
         <v>7598.96</v>
       </c>
-      <c r="C25" s="2" t="n">
+      <c r="C26" s="2" t="n">
         <v>752</v>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>-$6.91M</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>+$6.93M</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>7653.52</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>7600</v>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>-$5.45M</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>+$5.86M</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">

</xml_diff>